<commit_message>
Update master diamond inventory (7 stones) – 2026-09-08 09:26 UTC
</commit_message>
<xml_diff>
--- a/data/master_diamonds.xlsx
+++ b/data/master_diamonds.xlsx
@@ -637,11 +637,7 @@
           <t>EX</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>EX</t>

</xml_diff>

<commit_message>
Update master diamond inventory (17 stones) – 2026-09-08 09:27 UTC
</commit_message>
<xml_diff>
--- a/data/master_diamonds.xlsx
+++ b/data/master_diamonds.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -994,6 +994,644 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>10.97*7.86*5.16</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>11483.57</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>3.00 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>11.01*7.94*5.13</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>10856.48</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>3.00 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>10.88*7.92*5.16</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>11055</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>https://v360.in/diamondview.aspx?cid=LG2&amp;d=S-2417-1</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>3.00 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>10.22 x 7.42 x 4.86</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>9049.59</v>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>10.88 x 7.67 x 4.66</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>10588.37</v>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>10.64 x 7.62 x 4.50</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>9887.959999999999</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>10.90 x 7.69 x 4.68</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>10064.6</v>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>10.62 x 7.60 x 4.85</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>9890</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>video_link: DNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>9.48 x 6.07 x 3.78</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>3110</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>https://d1s5m21q2l18ke.cloudfront.net/v360_mov/j5jb5mjj235.HTML?sv=1&amp;displayAllSideview=1</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1.25 Pear  .xlsx</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>9.60 x 6.00 x 3.71</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>3840</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>https://v360.diamonds/u/813286ce-88fc-40b6-812e-1e46f48dd9d9?m=i</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1.25 Pear  .xlsx</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update master diamond inventory (17 stones) – 2026-09-08 10:08 UTC
</commit_message>
<xml_diff>
--- a/data/master_diamonds.xlsx
+++ b/data/master_diamonds.xlsx
@@ -46,8 +46,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -514,12 +515,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>OV3.00W913751</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>1535750439</t>
         </is>
@@ -589,12 +590,12 @@
       <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>OV2.50W918969</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>2547813803</t>
         </is>
@@ -660,12 +661,12 @@
       <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>OV2.50W918910</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>2546801653</t>
         </is>
@@ -735,8 +736,8 @@
       <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr"/>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>7558006636</t>
         </is>
@@ -800,8 +801,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr"/>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>1538847532</t>
         </is>
@@ -865,8 +866,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr"/>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>1543780240</t>
         </is>
@@ -930,8 +931,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr"/>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>7491630633</t>
         </is>
@@ -995,8 +996,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
+      <c r="A9" s="1" t="inlineStr"/>
+      <c r="B9" s="1" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1056,8 +1057,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
+      <c r="A10" s="1" t="inlineStr"/>
+      <c r="B10" s="1" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1117,8 +1118,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
+      <c r="A11" s="1" t="inlineStr"/>
+      <c r="B11" s="1" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1178,8 +1179,8 @@
       <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
+      <c r="A12" s="1" t="inlineStr"/>
+      <c r="B12" s="1" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1218,11 +1219,7 @@
           <t>EX</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
         <v>9049.59</v>
@@ -1243,8 +1240,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
+      <c r="A13" s="1" t="inlineStr"/>
+      <c r="B13" s="1" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1283,11 +1280,7 @@
           <t>EX</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>10588.37</v>
@@ -1308,8 +1301,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
+      <c r="A14" s="1" t="inlineStr"/>
+      <c r="B14" s="1" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1348,11 +1341,7 @@
           <t>EX</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
         <v>9887.959999999999</v>
@@ -1373,8 +1362,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
+      <c r="A15" s="1" t="inlineStr"/>
+      <c r="B15" s="1" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1413,11 +1402,7 @@
           <t>EX</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
         <v>10064.6</v>
@@ -1438,8 +1423,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
+      <c r="A16" s="1" t="inlineStr"/>
+      <c r="B16" s="1" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1478,11 +1463,7 @@
           <t>EX</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
         <v>9890</v>
@@ -1503,8 +1484,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="A17" s="1" t="inlineStr"/>
+      <c r="B17" s="1" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1543,11 +1524,7 @@
           <t>EX</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
         <v>3110</v>
@@ -1568,8 +1545,8 @@
       <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="A18" s="1" t="inlineStr"/>
+      <c r="B18" s="1" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>GIA</t>
@@ -1608,11 +1585,7 @@
           <t>EX</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
         <v>3840</v>

</xml_diff>

<commit_message>
Update master diamond inventory (79 stones) – 2026-09-08 10:27 UTC
</commit_message>
<xml_diff>
--- a/data/master_diamonds.xlsx
+++ b/data/master_diamonds.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S18"/>
+  <dimension ref="A1:S80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1605,6 +1605,4484 @@
       </c>
       <c r="S18" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr"/>
+      <c r="B19" s="1" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>9.32 x 5.92 x 3.84</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>VS1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>4959</v>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Mix.xlsx</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>video_link: Video; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr"/>
+      <c r="B20" s="1" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>9.90 x 6.08 x 3.80</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>VS1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>4465</v>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Mix.xlsx</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>video_link: Video; certificate_link: Pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr"/>
+      <c r="B21" s="1" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>10.16 x 6.50 x 3.85</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>VS1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>6681</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>https://d1wzmxdlubs910.cloudfront.net/VIDEOS/1951695.html</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Mix.xlsx</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr"/>
+      <c r="B22" s="1" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>9.87 x 6.25 x 4.03</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>5456</v>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Mix.xlsx</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>video_link: Video; certificate_link: Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr"/>
+      <c r="B23" s="1" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>9.88 x 6.33 x 3.96</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>VS1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>6137</v>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>https://media.mydiamonds.info/diamond-detail.aspx?r=ZSMKN169</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Mix.xlsx</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr"/>
+      <c r="B24" s="1" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>9.76 x 6.29 x 4.05</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>5256</v>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Mix.xlsx</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>video_link: Video; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>S26-8700</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>7551382216</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>5.06 - 5.09 * 3.18</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>892.5</v>
+      </c>
+      <c r="N25" t="n">
+        <v>446.25</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>S26-8849</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>1559419210</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>5.05 - 5.08 * 3.16</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>892.5</v>
+      </c>
+      <c r="N26" t="n">
+        <v>446.25</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>S26-9229</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>6552468665</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>5.10 - 5.13 * 3.13</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>881.25</v>
+      </c>
+      <c r="N27" t="n">
+        <v>440.63</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>S26-11189</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>6552783860</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>5.08 - 5.12 * 3.18</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>900</v>
+      </c>
+      <c r="N28" t="n">
+        <v>450</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>G26-15904</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>7546990830</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>5.07 - 5.10 * 3.16</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>900</v>
+      </c>
+      <c r="N29" t="n">
+        <v>450</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>G26-16874</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>5556105313</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>5.08 - 5.10 * 3.14</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M30" t="n">
+        <v>900</v>
+      </c>
+      <c r="N30" t="n">
+        <v>450</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>G26-17183</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>1558142571</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>5.05 - 5.09 * 3.14</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>892.5</v>
+      </c>
+      <c r="N31" t="n">
+        <v>446.25</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>G26-20084</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>2557480729</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>5.06 - 5.08 * 3.18</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>915</v>
+      </c>
+      <c r="N32" t="n">
+        <v>457.5</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>G26-25152</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>2564049910</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>5.05 - 5.08 * 3.15</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>900</v>
+      </c>
+      <c r="N33" t="n">
+        <v>450</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>G26-25803</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>1565088406</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>5.05 - 5.09 * 3.16</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>900</v>
+      </c>
+      <c r="N34" t="n">
+        <v>450</v>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>G26-24848</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>5563044561</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>5.09 - 5.12 * 3.11</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M35" t="n">
+        <v>885</v>
+      </c>
+      <c r="N35" t="n">
+        <v>442.5</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>G26-23042</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>6552871330</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>5.09 - 5.11 * 3.13</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>900</v>
+      </c>
+      <c r="N36" t="n">
+        <v>450</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>G26-20478</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>2557573270</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>5.12 - 5.16 * 3.06</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>888.75</v>
+      </c>
+      <c r="N37" t="n">
+        <v>444.38</v>
+      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>G26-19897</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>6555536723</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>5.09 - 5.13 * 3.13</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>907.5</v>
+      </c>
+      <c r="N38" t="n">
+        <v>453.75</v>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>G26-20275</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>2556543501</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>5.04 - 5.08 * 3.19</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>888.75</v>
+      </c>
+      <c r="N39" t="n">
+        <v>444.38</v>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>G26-20373</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>2557560004</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>5.08 - 5.10 * 3.19</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>960</v>
+      </c>
+      <c r="N40" t="n">
+        <v>480</v>
+      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>G26-20492</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>1558573482</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>5.03 - 5.07 * 3.18</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>900</v>
+      </c>
+      <c r="N41" t="n">
+        <v>450</v>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>G26-26253</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>7568101710</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>5.04 - 5.08 * 3.17</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>922.5</v>
+      </c>
+      <c r="N42" t="n">
+        <v>461.25</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>G26-22133</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>1555727471</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>5.06 - 5.09 * 3.15</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M43" t="n">
+        <v>915</v>
+      </c>
+      <c r="N43" t="n">
+        <v>457.5</v>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>G26-21785</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>1559704515</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>5.05 - 5.08 * 3.15</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>900</v>
+      </c>
+      <c r="N44" t="n">
+        <v>450</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>G26-22548</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>1559760740</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>5.05 - 5.08 * 3.18</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>900</v>
+      </c>
+      <c r="N45" t="n">
+        <v>450</v>
+      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>Z26-1849</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>7556408947</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>5.16 - 5.18 * 3.05</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>888.75</v>
+      </c>
+      <c r="N46" t="n">
+        <v>444.38</v>
+      </c>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>S26-6635</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>6541805834</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>5.04 - 5.11 * 3.14</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>817.5</v>
+      </c>
+      <c r="N47" t="n">
+        <v>408.75</v>
+      </c>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>G26-17179</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>6555146972</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>4.99 - 5.07 * 3.19</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>806.25</v>
+      </c>
+      <c r="N48" t="n">
+        <v>403.13</v>
+      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>G26-21727</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>6552699327</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>5.02 - 5.07 * 3.15</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>825</v>
+      </c>
+      <c r="N49" t="n">
+        <v>412.5</v>
+      </c>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>G26-24942</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>6551907309</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>5.02 - 5.06 * 3.16</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>847.5</v>
+      </c>
+      <c r="N50" t="n">
+        <v>423.75</v>
+      </c>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>G26-25828</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>1559998060</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>5.12 - 5.14 * 3.13</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M51" t="n">
+        <v>765</v>
+      </c>
+      <c r="N51" t="n">
+        <v>382.5</v>
+      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>S26-9352</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>7556482569</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>4.92 - 4.99 * 3.20</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>780</v>
+      </c>
+      <c r="N52" t="n">
+        <v>390</v>
+      </c>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>G26-20365</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>2558560854</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>4.96 - 5.01 * 3.21</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>795</v>
+      </c>
+      <c r="N53" t="n">
+        <v>397.5</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>G26-20611</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>1553591983</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>4.91 - 4.98 * 3.18</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>783.75</v>
+      </c>
+      <c r="N54" t="n">
+        <v>391.88</v>
+      </c>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>G26-25945</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>1569085465</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>4.96 - 5.01 * 3.18</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>810</v>
+      </c>
+      <c r="N55" t="n">
+        <v>405</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>G26-22161</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>2554712622</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>5.11 - 5.15 * 3.08</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>795</v>
+      </c>
+      <c r="N56" t="n">
+        <v>397.5</v>
+      </c>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>G26-22617</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>6555763963</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>4.99 - 5.04 * 3.18</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>810</v>
+      </c>
+      <c r="N57" t="n">
+        <v>405</v>
+      </c>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>G26-23850</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>2556954060</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>5.08 - 5.11 * 3.08</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>832.5</v>
+      </c>
+      <c r="N58" t="n">
+        <v>416.25</v>
+      </c>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>G26-25096</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>2566044074</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>4.95 - 5.00 * 3.18</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>795</v>
+      </c>
+      <c r="N59" t="n">
+        <v>397.5</v>
+      </c>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>G26-25485</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t>1568080703</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>5.07 - 5.09 * 3.19</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>900</v>
+      </c>
+      <c r="N60" t="n">
+        <v>459</v>
+      </c>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>G26-25185</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>6561048107</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>5.09 - 5.12 * 3.20</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>900</v>
+      </c>
+      <c r="N61" t="n">
+        <v>459</v>
+      </c>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>Z26-1730</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>1555473025</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>5.10 - 5.13 * 3.18</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>945</v>
+      </c>
+      <c r="N62" t="n">
+        <v>481.95</v>
+      </c>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>G26-24669</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>3555909277</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>5.13 - 5.16 * 3.18</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>907.5</v>
+      </c>
+      <c r="N63" t="n">
+        <v>471.9</v>
+      </c>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>G26-26417</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>5566019902</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>5.12 - 5.15 * 3.22</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M64" t="n">
+        <v>907.5</v>
+      </c>
+      <c r="N64" t="n">
+        <v>471.9</v>
+      </c>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>S26-9028</t>
+        </is>
+      </c>
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>7556443866</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>5.16 - 5.19 * 3.21</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>881.25</v>
+      </c>
+      <c r="N65" t="n">
+        <v>467.06</v>
+      </c>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>G26-25296</t>
+        </is>
+      </c>
+      <c r="B66" s="1" t="inlineStr">
+        <is>
+          <t>7568068922</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>5.16 - 5.19 * 3.21</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>915</v>
+      </c>
+      <c r="N66" t="n">
+        <v>484.95</v>
+      </c>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>G26-26252</t>
+        </is>
+      </c>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>2566101901</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>5.16 - 5.20 * 3.20</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>881.25</v>
+      </c>
+      <c r="N67" t="n">
+        <v>467.06</v>
+      </c>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="inlineStr">
+        <is>
+          <t>G26-22477</t>
+        </is>
+      </c>
+      <c r="B68" s="1" t="inlineStr">
+        <is>
+          <t>1553765377</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>5.25 - 5.28 * 3.15</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>892.5</v>
+      </c>
+      <c r="N68" t="n">
+        <v>473.03</v>
+      </c>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>G26-24760</t>
+        </is>
+      </c>
+      <c r="B69" s="1" t="inlineStr">
+        <is>
+          <t>2564024950</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>5.19 - 5.20 * 3.21</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>907.5</v>
+      </c>
+      <c r="N69" t="n">
+        <v>480.98</v>
+      </c>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>G26-16885</t>
+        </is>
+      </c>
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t>7551118098</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>5.21 - 5.22 * 3.27</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>862.5</v>
+      </c>
+      <c r="N70" t="n">
+        <v>465.75</v>
+      </c>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Data_2026-8-22_12-32-36.xlsx</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr"/>
+      <c r="B71" s="1" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>10.97*7.86*5.16</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="n">
+        <v>11483.57</v>
+      </c>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>3.00 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr"/>
+      <c r="B72" s="1" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>11.01*7.94*5.13</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="n">
+        <v>10856.48</v>
+      </c>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>3.00 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr"/>
+      <c r="B73" s="1" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>10.88*7.92*5.16</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>SI1</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="n">
+        <v>11055</v>
+      </c>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>https://v360.in/diamondview.aspx?cid=LG2&amp;d=S-2417-1</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>3.00 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr"/>
+      <c r="B74" s="1" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>10.22 x 7.42 x 4.86</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="n">
+        <v>9049.59</v>
+      </c>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr"/>
+      <c r="B75" s="1" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>10.88 x 7.67 x 4.66</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="n">
+        <v>10588.37</v>
+      </c>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr"/>
+      <c r="B76" s="1" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>10.64 x 7.62 x 4.50</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="n">
+        <v>9887.959999999999</v>
+      </c>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr"/>
+      <c r="B77" s="1" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>10.90 x 7.69 x 4.68</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="n">
+        <v>10064.6</v>
+      </c>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>video_link: HD; certificate_link: GIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="inlineStr"/>
+      <c r="B78" s="1" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Oval</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>10.62 x 7.60 x 4.85</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="n">
+        <v>9890</v>
+      </c>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>2.50 Oval  .xlsx</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>video_link: DNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="inlineStr"/>
+      <c r="B79" s="1" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>9.48 x 6.07 x 3.78</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="n">
+        <v>3110</v>
+      </c>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>https://d1s5m21q2l18ke.cloudfront.net/v360_mov/j5jb5mjj235.HTML?sv=1&amp;displayAllSideview=1</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>1.25 Pear  .xlsx</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="inlineStr"/>
+      <c r="B80" s="1" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>GIA</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Pear</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>9.60 x 6.00 x 3.71</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>VS2</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="n">
+        <v>3840</v>
+      </c>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>https://v360.diamonds/u/813286ce-88fc-40b6-812e-1e46f48dd9d9?m=i</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>1.25 Pear  .xlsx</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>